<commit_message>
Update organization master hierarchy
</commit_message>
<xml_diff>
--- a/Because-2.0/数据表/org_master.xlsx
+++ b/Because-2.0/数据表/org_master.xlsx
@@ -473,10 +473,10 @@
         <v/>
       </c>
       <c r="I2" t="str">
-        <v>01149,01001,01011,01029,01052,01070,01024,01040,01041,01025,01072,01074,01076,01012,01075,01150,01014,01069,01031,01017,01032,01071,01033,01015,01021,01037,01030,01018,01016,01042,01073,D0101,01026,01036,01065,01022,01045,01039,01028,01034,01019,01044,01035,01023,01027,01013,D0102,01098,01091,01100,01101,01083,01085,01095,01096,01080,01094,01097,01089,01078,01081,01082,01084,01087,01088,01090,01092,01099,01061,01077,01062,01086,D0103,01108,01107,01109,01110,01111,01114,01116,01106,01057,01148,01120,01115,01093,01147,01118,01113,01102,01059,01060,01058,01144,01119,01117,01105,01112,D0104,01132,01063,01129,01064,01067,01133,01134,01127,01125,01128,01136,01151,01122,01123,01126,01135,01131,01137,01145,01068,01121,D0105,01050,01055,01049,01143,01142,01139,01051,01054,01048,01056,01046,01047,01140,01138,D0106,01213,01208,01212,01231,01203,01235,01227,01220,01229,01237,01219,01204,01223,01226,01238,01222,01205,01201,01210,01221,01217,01211,01209,01233,01214,01232,01215,01216,01224,01218,01234,01236,01206,01228,D0108,01323,01310,01345,01319,01336,01344,01301,01331,01341,01335,01328,01324,01326,01311,01342,01338,01317,01309,01302,01343,01308,01314,01315,01322,01337,01313,01346,01305,01312,01307,01306,01332,01330,01329,01304,01303,01316,01339,01320,D0109,01146,D0107,01666,01005,01007,01006,01004,01003,01009,01010,01002,01008,01500,01600,01200,01999,01888,07002,06011,07013,07011,07001,07808,07809,07806,07021,07888,07999,D0601,08013,08011,08012,08015,08002,08888,08999,D0801,09002,09013,09015,09016,09012,09014,09011,09999,09888,D0901,10002,10011,10012,10013,10888,10999,D1001,11999,11001,11836,11846,11826,11808,11809,11005,11003,11002,11004,11816,11888,04888,04012,04011,04999,04002,D0401,D0501,05012,05011,05999,05888,05002,W0702,WD202,W1102,WD104,WD201,W0501,W0703,WD102,W0704,W0401,WD105,W1103,W0901,WD601,WD501,WD301,W1101,WD106,WD101,WD103,WD203,WD602,02999,02011,02001,02031,02021,02041,02888,02111,03999,03011,03032,03021,03888,03001,0100</v>
+        <v>FR001,FR002,FR003,0100</v>
       </c>
       <c r="J2" t="str">
-        <v>01149 科技金融团队；01001 常州分行营业部；01011 武进支行；01029 雪堰支行；01052 洛阳支行；01070 夏溪支行；01024 中天名园支行；01040 礼嘉支行；01041 坂上支行；01025 珑玥花园支行；01072 成章支行；01074 东安支行；01076 金鼎支行；01012 湖塘支行；01075 村前支行；01150 德禾豪景支行；01014 马杭支行；01069 嘉泽支行；01031 漕桥支行；01017 聚湖路支行；01032 太滆支行；01071 厚余支行；01033 南宅支行；01015 常武北路支行；01021 兴隆街支行；01037 常武北路支行；01030 潘家支行；01018 南都支行；01016 花园街支行；01042 政平支行；01073 湟里支行；D0101 武进支行大客户团队；01026 南夏墅支行；01036 运村支行；01065 礼河支行；01022 武宜路支行；01045 西太湖科技支行；01039 长安家园支行；01028 庙桥支行；01034 前黄支行；01019 大学城支行；01044 卢家巷支行；01035 寨桥支行；01023 武南路支行；01027 南塘支行；01013 武进高新区支行；D0102 武进高新区支行大客户团队；01098 云河路支行；01091 龙成支行；01100 孟河支行；01101 万绥支行；01083 汉江路支行；01085 大名城支行；01095 汤庄支行；01096 西夏墅支行；01080 龙虎塘支行；01094 罗溪支行；01097 浦河支行；01089 魏村支行；01078 三井支行；01081 新桥支行；01082 薛家支行；01084 吕墅支行；01087 太湖路支行；01088 春江支行；01090 百丈支行；01092 安家支行；01099 小河支行；01061 奔牛支行；01077 新北支行；01062 九里支行；01086 锦绣路支行；D0103 新北支行大客户团队；01108 雕庄支行；01107 公园路支行；01109 浦前支行；01110 万都商城支行；01111 中吴支行；01114 劳动中路支行；01116 青龙支行；01106 文化宫支行；01057 郑陆支行；01148 新城金郡支行；01120 青山桥支行；01115 兰陵支行；01093 龙湖香醍漫步支行；01147 紫荆支行；01118 翠竹支行；01113 和平路支行；01102 天宁支行；01059 焦溪支行；01060 三河口支行；01058 东青支行；01144 延陵路支行；01119 通江路支行；01117 红梅支行；01105 润德半岛支行；01112 茶山支行；D0104 天宁支行大客户团队；01132 金星支行；01063 邹区支行；01129 怀德路支行；01064 卜弋支行；01067 灯城支行；01133 新闸支行；01134 冶金支行；01127 飞龙桥支行；01125 北港支行；01128 永红支行；01136 东岱支行；01151 凌家塘支行；01122 五星支行；01123 金色新城支行；01126 勤业支行；01135 城西支行；01131 荆川支行；01137 西林支行；01145 北大街支行；01068 邹新支行；01121 钟楼支行；D0105 钟楼支行大客户团队；01050 遥观支行；01055 芙蓉支行；01049 崔丰支行；01143 荷花苑支行；01142 剑湖支行；01139 御河湾花园支行；01051 塘桥支行；01054 横山桥支行；01048 崔桥支行；01056 新安支行；01046 横林支行；01047 横林镇南支行；01140 潞城支行；01138 经济开发区支行；D0106 经济开发区支行大客户团队；01213 金东支行；01208 华兴支行；01212 金虹支行；01231 西阳支行；01203 金江苑支行；01235 尧塘支行；01227 朱林支行；01220 五叶支行；01229 清华园支行；01237 水北支行；01219 儒林支行；01204 华城支行；01223 社头支行；01226 登冠支行；01238 岸头支行；01222 指前支行；01205 金沙支行；01201 金坛支行；01210 丹阳门支行；01221 东园支行；01217 金西支行；01211 东环支行；01209 虹翠支行；01233 花山支行；01214 后阳支行；01232 茅麓支行；01215 南洲花园支行；01216 小南门支行；01224 直溪支行；01218 中塘支行；01234 罗村支行；01236 南汤支行；01206 白塔支行；01228 西岗支行；D0108 金坛市支行大客户团队；01323 后六支行；01310 平陵支行；01345 周城支行；01319 燕山支行；01336 上兴支行；01344 社渚支行；01301 溧阳市支行；01331 屏峰支行；01341 强埠支行；01335 后周支行；01328 天目湖支行；01324 上黄支行；01326 横涧支行；01311 西苑支行；01342 旧县支行；01338 竹箦支行；01317 西郊支行；01309 燕苑支行；01302 溧城支行；01343 联盟支行；01308 锦绣支行；01314 马垫支行；01315 杨庄支行；01322 埭头支行；01337 上沛支行；01313 江苏中关村科技支行；01346 振兴支行；01305 清安支行；01312 昆仑支行；01307 中兴支行；01306 泓口支行；01332 别桥支行；01330 平桥支行；01329 茶亭支行；01304 溧阳市城南支行；01303 溧阳市城中支行；01316 龙亭支行；01339 前马支行；01320 北大街支行；D0109 溧阳市支行大客户团队；01146 科技金融事业部；D0107 科技金融事业部大客户团队；01666 常州分行行长室；01005 常州分行信贷部；01007 常州分行合规部；01006 常州分行公司部；01004 常州分行资金部；01003 单证中心；01009 常州分行三农部；01010 常州分行运管部；01002 常州分行计财部；01008 常州分行风管部；01500 武进库区；01600 溧阳库区；01200 武进库区；01999 常州分行管理机构；01888 常州分行清算中心；07002 淮安分行财务部；06011 涟水支行；07013 淮安山阳分理处；07011 淮安区支行；07001 淮安分行营业部；07808 淮安分行风险部；07809 淮安分行零售部；07806 淮安分行公司部；07021 淮阴支行；07888 淮安分行清算中心；07999 淮安分行管理机构；D0601 涟水支行营业部大客户团队；08013 丹阳皇塘支行；08011 丹阳支行；08012 丹阳经济开发区支行；08015 丹阳丹北支行；08002 丹阳支行财务部；08888 丹阳支行清算中心；08999 丹阳支行管理机构；D0801 丹阳支行营业部大客户团队；09002 宜兴支行财务部；09013 宜兴官林分理处；09015 宜兴张渚分理处；09016 宜兴和桥分理处；09012 宜兴丁蜀分理处；09014 宜兴支行分理处；09011 宜兴支行；09999 宜兴支行管理机构；09888 宜兴支行清算中心；D0901 宜兴支行营业部大客户团队；10002 靖江支行财务部；10011 靖江支行；10012 靖江虹桥支行；10013 靖江城东支行；10888 靖江支行清算中心；10999 靖江支行管理机构；D1001 靖江支行营业部大客户团队；11999 苏州分行管理机构；11001 苏州分行；11836 苏州分行公司三部；11846 苏州分行公司四部；11826 苏州分行公司二部；11808 苏州分行风险部；11809 苏州分行零售部；11005 苏州张家港支行；11003 苏州吴中支行；11002 苏州分行财务部；11004 苏州常熟支行；11816 苏州分行公司一部；11888 苏州分行清算中心；04888 赣榆支行清算中心；04012 赣榆新城支行；04011 赣榆支行；04999 赣榆支行管理机构；04002 赣榆支行财务部；D0401 赣榆支行营业部大客户团队；D0501 东台支行营业部大客户团队；05012 东台御珑湾支行；05011 东台支行；05999 东台支行管理机构；05888 东台支行清算中心；05002 东台支行财务部；W0702 小微贷款事业部淮安营业部二队；WD202 小微贷款事业部小河团队（万绥）；W1102 小微贷款事业部张家港团队；WD104 小微贷款事业部郑陆团队（崔桥）；WD201 小微贷款事业部小河团队；W0501 小微贷款事业部东台团队；W0703 小微贷款事业部涟水团队；WD102 小微贷款事业部营业部团队；W0704 小微贷款事业部淮阴团队；W0401 小微贷款事业部赣榆团队；WD105 小微贷款事业部营业部团队（遥观）；W1103 小微贷款事业部苏州园区团队；W0901 小微贷款事业部宜兴团队；WD601 小微贷款事业部溧阳一队；WD501 小微贷款事业部金坛团队；WD301 小微贷款事业部郑陆团队；W1101 小微贷款事业部常熟团队；WD106 小微贷款事业部雪堰团队（坂上）；WD101 小微贷款事业部雪堰团队；WD103 小微贷款事业部湟里团队；WD203 小微贷款事业部小河团队（魏村）；WD602 小微贷款事业部溧阳二队；02999 大丰村镇银行管理机构；02011 大丰港支行；02001 江苏大丰江南村镇银行股份有限公司；02031 裕华支行；02021 刘庄支行；02041 健康西路支行；02888 大丰村镇银行清算中心；02111 大丰小微贷款事业部；03999 上海浦东江南村镇银行管理机构；03011 南汇支行；03032 普惠金融部团队；03021 三林支行；03888 上海浦东江南村镇银行清算中心；03001 上海浦东江南村镇银行营业部；0100 日终专用机构 (特殊节点，无下级)</v>
+        <v>FR001 江苏江南农村商业银行总行 (总行级)；FR002 大丰村镇银行 (独立法人)；FR003 上海浦东江南村镇银行 (独立法人)；0100 日终专用机构 (特殊节点，无下级)</v>
       </c>
       <c r="K2" t="str">
         <v/>
@@ -488,7 +488,7 @@
         <v>org_code='00000'</v>
       </c>
       <c r="N2" t="str">
-        <v>org_code IN ('01149','01001','01011','01029','01052','01070','01024','01040','01041','01025','01072','01074','01076','01012','01075','01150','01014','01069','01031','01017','01032','01071','01033','01015','01021','01037','01030','01018','01016','01042','01073','D0101','01026','01036','01065','01022','01045','01039','01028','01034','01019','01044','01035','01023','01027','01013','D0102','01098','01091','01100','01101','01083','01085','01095','01096','01080','01094','01097','01089','01078','01081','01082','01084','01087','01088','01090','01092','01099','01061','01077','01062','01086','D0103','01108','01107','01109','01110','01111','01114','01116','01106','01057','01148','01120','01115','01093','01147','01118','01113','01102','01059','01060','01058','01144','01119','01117','01105','01112','D0104','01132','01063','01129','01064','01067','01133','01134','01127','01125','01128','01136','01151','01122','01123','01126','01135','01131','01137','01145','01068','01121','D0105','01050','01055','01049','01143','01142','01139','01051','01054','01048','01056','01046','01047','01140','01138','D0106','01213','01208','01212','01231','01203','01235','01227','01220','01229','01237','01219','01204','01223','01226','01238','01222','01205','01201','01210','01221','01217','01211','01209','01233','01214','01232','01215','01216','01224','01218','01234','01236','01206','01228','D0108','01323','01310','01345','01319','01336','01344','01301','01331','01341','01335','01328','01324','01326','01311','01342','01338','01317','01309','01302','01343','01308','01314','01315','01322','01337','01313','01346','01305','01312','01307','01306','01332','01330','01329','01304','01303','01316','01339','01320','D0109','01146','D0107','01666','01005','01007','01006','01004','01003','01009','01010','01002','01008','01500','01600','01200','01999','01888','07002','06011','07013','07011','07001','07808','07809','07806','07021','07888','07999','D0601','08013','08011','08012','08015','08002','08888','08999','D0801','09002','09013','09015','09016','09012','09014','09011','09999','09888','D0901','10002','10011','10012','10013','10888','10999','D1001','11999','11001','11836','11846','11826','11808','11809','11005','11003','11002','11004','11816','11888','04888','04012','04011','04999','04002','D0401','D0501','05012','05011','05999','05888','05002','W0702','WD202','W1102','WD104','WD201','W0501','W0703','WD102','W0704','W0401','WD105','W1103','W0901','WD601','WD501','WD301','W1101','WD106','WD101','WD103','WD203','WD602','02999','02011','02001','02031','02021','02041','02888','02111','03999','03011','03032','03021','03888','03001','0100')</v>
+        <v>org_code IN ('FR001','FR002','FR003','0100')</v>
       </c>
       <c r="O2" t="str">
         <v/>
@@ -520,10 +520,10 @@
         <v/>
       </c>
       <c r="I3" t="str">
-        <v>01149,01001,01011,01029,01052,01070,01024,01040,01041,01025,01072,01074,01076,01012,01075,01150,01014,01069,01031,01017,01032,01071,01033,01015,01021,01037,01030,01018,01016,01042,01073,D0101,01026,01036,01065,01022,01045,01039,01028,01034,01019,01044,01035,01023,01027,01013,D0102,01098,01091,01100,01101,01083,01085,01095,01096,01080,01094,01097,01089,01078,01081,01082,01084,01087,01088,01090,01092,01099,01061,01077,01062,01086,D0103,01108,01107,01109,01110,01111,01114,01116,01106,01057,01148,01120,01115,01093,01147,01118,01113,01102,01059,01060,01058,01144,01119,01117,01105,01112,D0104,01132,01063,01129,01064,01067,01133,01134,01127,01125,01128,01136,01151,01122,01123,01126,01135,01131,01137,01145,01068,01121,D0105,01050,01055,01049,01143,01142,01139,01051,01054,01048,01056,01046,01047,01140,01138,D0106,01213,01208,01212,01231,01203,01235,01227,01220,01229,01237,01219,01204,01223,01226,01238,01222,01205,01201,01210,01221,01217,01211,01209,01233,01214,01232,01215,01216,01224,01218,01234,01236,01206,01228,D0108,01323,01310,01345,01319,01336,01344,01301,01331,01341,01335,01328,01324,01326,01311,01342,01338,01317,01309,01302,01343,01308,01314,01315,01322,01337,01313,01346,01305,01312,01307,01306,01332,01330,01329,01304,01303,01316,01339,01320,D0109,01146,D0107,01666,01005,01007,01006,01004,01003,01009,01010,01002,01008,01500,01600,01200,01999,01888,07002,06011,07013,07011,07001,07808,07809,07806,07021,07888,07999,D0601,08013,08011,08012,08015,08002,08888,08999,D0801,09002,09013,09015,09016,09012,09014,09011,09999,09888,D0901,10002,10011,10012,10013,10888,10999,D1001,11999,11001,11836,11846,11826,11808,11809,11005,11003,11002,11004,11816,11888,04888,04012,04011,04999,04002,D0401,D0501,05012,05011,05999,05888,05002,W0702,WD202,W1102,WD104,WD201,W0501,W0703,WD102,W0704,W0401,WD105,W1103,W0901,WD601,WD501,WD301,W1101,WD106,WD101,WD103,WD203,WD602</v>
+        <v>A8000,A0000,A0700,A0800,A0900,A1000,A1100,A0400,A0500,80041</v>
       </c>
       <c r="J3" t="str">
-        <v>01149 科技金融团队；01001 常州分行营业部；01011 武进支行；01029 雪堰支行；01052 洛阳支行；01070 夏溪支行；01024 中天名园支行；01040 礼嘉支行；01041 坂上支行；01025 珑玥花园支行；01072 成章支行；01074 东安支行；01076 金鼎支行；01012 湖塘支行；01075 村前支行；01150 德禾豪景支行；01014 马杭支行；01069 嘉泽支行；01031 漕桥支行；01017 聚湖路支行；01032 太滆支行；01071 厚余支行；01033 南宅支行；01015 常武北路支行；01021 兴隆街支行；01037 常武北路支行；01030 潘家支行；01018 南都支行；01016 花园街支行；01042 政平支行；01073 湟里支行；D0101 武进支行大客户团队；01026 南夏墅支行；01036 运村支行；01065 礼河支行；01022 武宜路支行；01045 西太湖科技支行；01039 长安家园支行；01028 庙桥支行；01034 前黄支行；01019 大学城支行；01044 卢家巷支行；01035 寨桥支行；01023 武南路支行；01027 南塘支行；01013 武进高新区支行；D0102 武进高新区支行大客户团队；01098 云河路支行；01091 龙成支行；01100 孟河支行；01101 万绥支行；01083 汉江路支行；01085 大名城支行；01095 汤庄支行；01096 西夏墅支行；01080 龙虎塘支行；01094 罗溪支行；01097 浦河支行；01089 魏村支行；01078 三井支行；01081 新桥支行；01082 薛家支行；01084 吕墅支行；01087 太湖路支行；01088 春江支行；01090 百丈支行；01092 安家支行；01099 小河支行；01061 奔牛支行；01077 新北支行；01062 九里支行；01086 锦绣路支行；D0103 新北支行大客户团队；01108 雕庄支行；01107 公园路支行；01109 浦前支行；01110 万都商城支行；01111 中吴支行；01114 劳动中路支行；01116 青龙支行；01106 文化宫支行；01057 郑陆支行；01148 新城金郡支行；01120 青山桥支行；01115 兰陵支行；01093 龙湖香醍漫步支行；01147 紫荆支行；01118 翠竹支行；01113 和平路支行；01102 天宁支行；01059 焦溪支行；01060 三河口支行；01058 东青支行；01144 延陵路支行；01119 通江路支行；01117 红梅支行；01105 润德半岛支行；01112 茶山支行；D0104 天宁支行大客户团队；01132 金星支行；01063 邹区支行；01129 怀德路支行；01064 卜弋支行；01067 灯城支行；01133 新闸支行；01134 冶金支行；01127 飞龙桥支行；01125 北港支行；01128 永红支行；01136 东岱支行；01151 凌家塘支行；01122 五星支行；01123 金色新城支行；01126 勤业支行；01135 城西支行；01131 荆川支行；01137 西林支行；01145 北大街支行；01068 邹新支行；01121 钟楼支行；D0105 钟楼支行大客户团队；01050 遥观支行；01055 芙蓉支行；01049 崔丰支行；01143 荷花苑支行；01142 剑湖支行；01139 御河湾花园支行；01051 塘桥支行；01054 横山桥支行；01048 崔桥支行；01056 新安支行；01046 横林支行；01047 横林镇南支行；01140 潞城支行；01138 经济开发区支行；D0106 经济开发区支行大客户团队；01213 金东支行；01208 华兴支行；01212 金虹支行；01231 西阳支行；01203 金江苑支行；01235 尧塘支行；01227 朱林支行；01220 五叶支行；01229 清华园支行；01237 水北支行；01219 儒林支行；01204 华城支行；01223 社头支行；01226 登冠支行；01238 岸头支行；01222 指前支行；01205 金沙支行；01201 金坛支行；01210 丹阳门支行；01221 东园支行；01217 金西支行；01211 东环支行；01209 虹翠支行；01233 花山支行；01214 后阳支行；01232 茅麓支行；01215 南洲花园支行；01216 小南门支行；01224 直溪支行；01218 中塘支行；01234 罗村支行；01236 南汤支行；01206 白塔支行；01228 西岗支行；D0108 金坛市支行大客户团队；01323 后六支行；01310 平陵支行；01345 周城支行；01319 燕山支行；01336 上兴支行；01344 社渚支行；01301 溧阳市支行；01331 屏峰支行；01341 强埠支行；01335 后周支行；01328 天目湖支行；01324 上黄支行；01326 横涧支行；01311 西苑支行；01342 旧县支行；01338 竹箦支行；01317 西郊支行；01309 燕苑支行；01302 溧城支行；01343 联盟支行；01308 锦绣支行；01314 马垫支行；01315 杨庄支行；01322 埭头支行；01337 上沛支行；01313 江苏中关村科技支行；01346 振兴支行；01305 清安支行；01312 昆仑支行；01307 中兴支行；01306 泓口支行；01332 别桥支行；01330 平桥支行；01329 茶亭支行；01304 溧阳市城南支行；01303 溧阳市城中支行；01316 龙亭支行；01339 前马支行；01320 北大街支行；D0109 溧阳市支行大客户团队；01146 科技金融事业部；D0107 科技金融事业部大客户团队；01666 常州分行行长室；01005 常州分行信贷部；01007 常州分行合规部；01006 常州分行公司部；01004 常州分行资金部；01003 单证中心；01009 常州分行三农部；01010 常州分行运管部；01002 常州分行计财部；01008 常州分行风管部；01500 武进库区；01600 溧阳库区；01200 武进库区；01999 常州分行管理机构；01888 常州分行清算中心；07002 淮安分行财务部；06011 涟水支行；07013 淮安山阳分理处；07011 淮安区支行；07001 淮安分行营业部；07808 淮安分行风险部；07809 淮安分行零售部；07806 淮安分行公司部；07021 淮阴支行；07888 淮安分行清算中心；07999 淮安分行管理机构；D0601 涟水支行营业部大客户团队；08013 丹阳皇塘支行；08011 丹阳支行；08012 丹阳经济开发区支行；08015 丹阳丹北支行；08002 丹阳支行财务部；08888 丹阳支行清算中心；08999 丹阳支行管理机构；D0801 丹阳支行营业部大客户团队；09002 宜兴支行财务部；09013 宜兴官林分理处；09015 宜兴张渚分理处；09016 宜兴和桥分理处；09012 宜兴丁蜀分理处；09014 宜兴支行分理处；09011 宜兴支行；09999 宜兴支行管理机构；09888 宜兴支行清算中心；D0901 宜兴支行营业部大客户团队；10002 靖江支行财务部；10011 靖江支行；10012 靖江虹桥支行；10013 靖江城东支行；10888 靖江支行清算中心；10999 靖江支行管理机构；D1001 靖江支行营业部大客户团队；11999 苏州分行管理机构；11001 苏州分行；11836 苏州分行公司三部；11846 苏州分行公司四部；11826 苏州分行公司二部；11808 苏州分行风险部；11809 苏州分行零售部；11005 苏州张家港支行；11003 苏州吴中支行；11002 苏州分行财务部；11004 苏州常熟支行；11816 苏州分行公司一部；11888 苏州分行清算中心；04888 赣榆支行清算中心；04012 赣榆新城支行；04011 赣榆支行；04999 赣榆支行管理机构；04002 赣榆支行财务部；D0401 赣榆支行营业部大客户团队；D0501 东台支行营业部大客户团队；05012 东台御珑湾支行；05011 东台支行；05999 东台支行管理机构；05888 东台支行清算中心；05002 东台支行财务部；W0702 小微贷款事业部淮安营业部二队；WD202 小微贷款事业部小河团队（万绥）；W1102 小微贷款事业部张家港团队；WD104 小微贷款事业部郑陆团队（崔桥）；WD201 小微贷款事业部小河团队；W0501 小微贷款事业部东台团队；W0703 小微贷款事业部涟水团队；WD102 小微贷款事业部营业部团队；W0704 小微贷款事业部淮阴团队；W0401 小微贷款事业部赣榆团队；WD105 小微贷款事业部营业部团队（遥观）；W1103 小微贷款事业部苏州园区团队；W0901 小微贷款事业部宜兴团队；WD601 小微贷款事业部溧阳一队；WD501 小微贷款事业部金坛团队；WD301 小微贷款事业部郑陆团队；W1101 小微贷款事业部常熟团队；WD106 小微贷款事业部雪堰团队（坂上）；WD101 小微贷款事业部雪堰团队；WD103 小微贷款事业部湟里团队；WD203 小微贷款事业部小河团队（魏村）；WD602 小微贷款事业部溧阳二队</v>
+        <v>A8000 总行部室；A0000 常州分行；A0700 淮安分行；A0800 丹阳支行；A0900 宜兴支行；A1000 靖江支行；A1100 苏州分行；A0400 赣榆支行；A0500 东台支行；80041 江南农商行小微贷款事业部</v>
       </c>
       <c r="K3" t="str">
         <v>FR001,FR002,FR003</v>
@@ -535,7 +535,7 @@
         <v>org_code='FR001'</v>
       </c>
       <c r="N3" t="str">
-        <v>org_code IN ('01149','01001','01011','01029','01052','01070','01024','01040','01041','01025','01072','01074','01076','01012','01075','01150','01014','01069','01031','01017','01032','01071','01033','01015','01021','01037','01030','01018','01016','01042','01073','D0101','01026','01036','01065','01022','01045','01039','01028','01034','01019','01044','01035','01023','01027','01013','D0102','01098','01091','01100','01101','01083','01085','01095','01096','01080','01094','01097','01089','01078','01081','01082','01084','01087','01088','01090','01092','01099','01061','01077','01062','01086','D0103','01108','01107','01109','01110','01111','01114','01116','01106','01057','01148','01120','01115','01093','01147','01118','01113','01102','01059','01060','01058','01144','01119','01117','01105','01112','D0104','01132','01063','01129','01064','01067','01133','01134','01127','01125','01128','01136','01151','01122','01123','01126','01135','01131','01137','01145','01068','01121','D0105','01050','01055','01049','01143','01142','01139','01051','01054','01048','01056','01046','01047','01140','01138','D0106','01213','01208','01212','01231','01203','01235','01227','01220','01229','01237','01219','01204','01223','01226','01238','01222','01205','01201','01210','01221','01217','01211','01209','01233','01214','01232','01215','01216','01224','01218','01234','01236','01206','01228','D0108','01323','01310','01345','01319','01336','01344','01301','01331','01341','01335','01328','01324','01326','01311','01342','01338','01317','01309','01302','01343','01308','01314','01315','01322','01337','01313','01346','01305','01312','01307','01306','01332','01330','01329','01304','01303','01316','01339','01320','D0109','01146','D0107','01666','01005','01007','01006','01004','01003','01009','01010','01002','01008','01500','01600','01200','01999','01888','07002','06011','07013','07011','07001','07808','07809','07806','07021','07888','07999','D0601','08013','08011','08012','08015','08002','08888','08999','D0801','09002','09013','09015','09016','09012','09014','09011','09999','09888','D0901','10002','10011','10012','10013','10888','10999','D1001','11999','11001','11836','11846','11826','11808','11809','11005','11003','11002','11004','11816','11888','04888','04012','04011','04999','04002','D0401','D0501','05012','05011','05999','05888','05002','W0702','WD202','W1102','WD104','WD201','W0501','W0703','WD102','W0704','W0401','WD105','W1103','W0901','WD601','WD501','WD301','W1101','WD106','WD101','WD103','WD203','WD602')</v>
+        <v>org_code IN ('A8000','A0000','A0700','A0800','A0900','A1000','A1100','A0400','A0500','80041')</v>
       </c>
       <c r="O3" t="str">
         <v/>
@@ -614,10 +614,10 @@
         <v>区域权限：常州全辖</v>
       </c>
       <c r="I5" t="str">
-        <v>01149,01001,01011,01029,01052,01070,01024,01040,01041,01025,01072,01074,01076,01012,01075,01150,01014,01069,01031,01017,01032,01071,01033,01015,01021,01037,01030,01018,01016,01042,01073,D0101,01026,01036,01065,01022,01045,01039,01028,01034,01019,01044,01035,01023,01027,01013,D0102,01098,01091,01100,01101,01083,01085,01095,01096,01080,01094,01097,01089,01078,01081,01082,01084,01087,01088,01090,01092,01099,01061,01077,01062,01086,D0103,01108,01107,01109,01110,01111,01114,01116,01106,01057,01148,01120,01115,01093,01147,01118,01113,01102,01059,01060,01058,01144,01119,01117,01105,01112,D0104,01132,01063,01129,01064,01067,01133,01134,01127,01125,01128,01136,01151,01122,01123,01126,01135,01131,01137,01145,01068,01121,D0105,01050,01055,01049,01143,01142,01139,01051,01054,01048,01056,01046,01047,01140,01138,D0106,01213,01208,01212,01231,01203,01235,01227,01220,01229,01237,01219,01204,01223,01226,01238,01222,01205,01201,01210,01221,01217,01211,01209,01233,01214,01232,01215,01216,01224,01218,01234,01236,01206,01228,D0108,01323,01310,01345,01319,01336,01344,01301,01331,01341,01335,01328,01324,01326,01311,01342,01338,01317,01309,01302,01343,01308,01314,01315,01322,01337,01313,01346,01305,01312,01307,01306,01332,01330,01329,01304,01303,01316,01339,01320,D0109,01146,D0107,01666,01005,01007,01006,01004,01003,01009,01010,01002,01008,01500,01600,01200,01999,01888</v>
+        <v>A0001,A0002,A0003,A0004,A0005,A0006,A0007,A0008,A0009,A0010</v>
       </c>
       <c r="J5" t="str">
-        <v>01149 科技金融团队；01001 常州分行营业部；01011 武进支行；01029 雪堰支行；01052 洛阳支行；01070 夏溪支行；01024 中天名园支行；01040 礼嘉支行；01041 坂上支行；01025 珑玥花园支行；01072 成章支行；01074 东安支行；01076 金鼎支行；01012 湖塘支行；01075 村前支行；01150 德禾豪景支行；01014 马杭支行；01069 嘉泽支行；01031 漕桥支行；01017 聚湖路支行；01032 太滆支行；01071 厚余支行；01033 南宅支行；01015 常武北路支行；01021 兴隆街支行；01037 常武北路支行；01030 潘家支行；01018 南都支行；01016 花园街支行；01042 政平支行；01073 湟里支行；D0101 武进支行大客户团队；01026 南夏墅支行；01036 运村支行；01065 礼河支行；01022 武宜路支行；01045 西太湖科技支行；01039 长安家园支行；01028 庙桥支行；01034 前黄支行；01019 大学城支行；01044 卢家巷支行；01035 寨桥支行；01023 武南路支行；01027 南塘支行；01013 武进高新区支行；D0102 武进高新区支行大客户团队；01098 云河路支行；01091 龙成支行；01100 孟河支行；01101 万绥支行；01083 汉江路支行；01085 大名城支行；01095 汤庄支行；01096 西夏墅支行；01080 龙虎塘支行；01094 罗溪支行；01097 浦河支行；01089 魏村支行；01078 三井支行；01081 新桥支行；01082 薛家支行；01084 吕墅支行；01087 太湖路支行；01088 春江支行；01090 百丈支行；01092 安家支行；01099 小河支行；01061 奔牛支行；01077 新北支行；01062 九里支行；01086 锦绣路支行；D0103 新北支行大客户团队；01108 雕庄支行；01107 公园路支行；01109 浦前支行；01110 万都商城支行；01111 中吴支行；01114 劳动中路支行；01116 青龙支行；01106 文化宫支行；01057 郑陆支行；01148 新城金郡支行；01120 青山桥支行；01115 兰陵支行；01093 龙湖香醍漫步支行；01147 紫荆支行；01118 翠竹支行；01113 和平路支行；01102 天宁支行；01059 焦溪支行；01060 三河口支行；01058 东青支行；01144 延陵路支行；01119 通江路支行；01117 红梅支行；01105 润德半岛支行；01112 茶山支行；D0104 天宁支行大客户团队；01132 金星支行；01063 邹区支行；01129 怀德路支行；01064 卜弋支行；01067 灯城支行；01133 新闸支行；01134 冶金支行；01127 飞龙桥支行；01125 北港支行；01128 永红支行；01136 东岱支行；01151 凌家塘支行；01122 五星支行；01123 金色新城支行；01126 勤业支行；01135 城西支行；01131 荆川支行；01137 西林支行；01145 北大街支行；01068 邹新支行；01121 钟楼支行；D0105 钟楼支行大客户团队；01050 遥观支行；01055 芙蓉支行；01049 崔丰支行；01143 荷花苑支行；01142 剑湖支行；01139 御河湾花园支行；01051 塘桥支行；01054 横山桥支行；01048 崔桥支行；01056 新安支行；01046 横林支行；01047 横林镇南支行；01140 潞城支行；01138 经济开发区支行；D0106 经济开发区支行大客户团队；01213 金东支行；01208 华兴支行；01212 金虹支行；01231 西阳支行；01203 金江苑支行；01235 尧塘支行；01227 朱林支行；01220 五叶支行；01229 清华园支行；01237 水北支行；01219 儒林支行；01204 华城支行；01223 社头支行；01226 登冠支行；01238 岸头支行；01222 指前支行；01205 金沙支行；01201 金坛支行；01210 丹阳门支行；01221 东园支行；01217 金西支行；01211 东环支行；01209 虹翠支行；01233 花山支行；01214 后阳支行；01232 茅麓支行；01215 南洲花园支行；01216 小南门支行；01224 直溪支行；01218 中塘支行；01234 罗村支行；01236 南汤支行；01206 白塔支行；01228 西岗支行；D0108 金坛市支行大客户团队；01323 后六支行；01310 平陵支行；01345 周城支行；01319 燕山支行；01336 上兴支行；01344 社渚支行；01301 溧阳市支行；01331 屏峰支行；01341 强埠支行；01335 后周支行；01328 天目湖支行；01324 上黄支行；01326 横涧支行；01311 西苑支行；01342 旧县支行；01338 竹箦支行；01317 西郊支行；01309 燕苑支行；01302 溧城支行；01343 联盟支行；01308 锦绣支行；01314 马垫支行；01315 杨庄支行；01322 埭头支行；01337 上沛支行；01313 江苏中关村科技支行；01346 振兴支行；01305 清安支行；01312 昆仑支行；01307 中兴支行；01306 泓口支行；01332 别桥支行；01330 平桥支行；01329 茶亭支行；01304 溧阳市城南支行；01303 溧阳市城中支行；01316 龙亭支行；01339 前马支行；01320 北大街支行；D0109 溧阳市支行大客户团队；01146 科技金融事业部；D0107 科技金融事业部大客户团队；01666 常州分行行长室；01005 常州分行信贷部；01007 常州分行合规部；01006 常州分行公司部；01004 常州分行资金部；01003 单证中心；01009 常州分行三农部；01010 常州分行运管部；01002 常州分行计财部；01008 常州分行风管部；01500 武进库区；01600 溧阳库区；01200 武进库区；01999 常州分行管理机构；01888 常州分行清算中心</v>
+        <v>A0001 常州分行营业部；A0002 武进支行；A0003 武进高新区支行；A0004 新北支行；A0005 天宁支行；A0006 钟楼支行；A0007 经济开发区支行；A0008 金坛支行；A0009 溧阳市支行；A0010 科技金融事业部</v>
       </c>
       <c r="K5" t="str">
         <v>A0000,A0700,A0800,A0900,A1000,A1100,A0400,A0500</v>
@@ -629,7 +629,7 @@
         <v>org_code='A0000'</v>
       </c>
       <c r="N5" t="str">
-        <v>org_code IN ('01149','01001','01011','01029','01052','01070','01024','01040','01041','01025','01072','01074','01076','01012','01075','01150','01014','01069','01031','01017','01032','01071','01033','01015','01021','01037','01030','01018','01016','01042','01073','D0101','01026','01036','01065','01022','01045','01039','01028','01034','01019','01044','01035','01023','01027','01013','D0102','01098','01091','01100','01101','01083','01085','01095','01096','01080','01094','01097','01089','01078','01081','01082','01084','01087','01088','01090','01092','01099','01061','01077','01062','01086','D0103','01108','01107','01109','01110','01111','01114','01116','01106','01057','01148','01120','01115','01093','01147','01118','01113','01102','01059','01060','01058','01144','01119','01117','01105','01112','D0104','01132','01063','01129','01064','01067','01133','01134','01127','01125','01128','01136','01151','01122','01123','01126','01135','01131','01137','01145','01068','01121','D0105','01050','01055','01049','01143','01142','01139','01051','01054','01048','01056','01046','01047','01140','01138','D0106','01213','01208','01212','01231','01203','01235','01227','01220','01229','01237','01219','01204','01223','01226','01238','01222','01205','01201','01210','01221','01217','01211','01209','01233','01214','01232','01215','01216','01224','01218','01234','01236','01206','01228','D0108','01323','01310','01345','01319','01336','01344','01301','01331','01341','01335','01328','01324','01326','01311','01342','01338','01317','01309','01302','01343','01308','01314','01315','01322','01337','01313','01346','01305','01312','01307','01306','01332','01330','01329','01304','01303','01316','01339','01320','D0109','01146','D0107','01666','01005','01007','01006','01004','01003','01009','01010','01002','01008','01500','01600','01200','01999','01888')</v>
+        <v>org_code IN ('A0001','A0002','A0003','A0004','A0005','A0006','A0007','A0008','A0009','A0010')</v>
       </c>
       <c r="O5" t="str">
         <v/>
@@ -11894,10 +11894,10 @@
         <v>区域权限：淮安全辖</v>
       </c>
       <c r="I245" t="str">
-        <v>07002,06011,07013,07011,07001,07808,07809,07806,07021,07888,07999,D0601</v>
+        <v>07002,06011,07013,07011,07001,07808,07809,07806,07021,07888,07999,A0701,A0702,A0703,D0601</v>
       </c>
       <c r="J245" t="str">
-        <v>07002 淮安分行财务部；06011 涟水支行；07013 淮安山阳分理处；07011 淮安区支行；07001 淮安分行营业部；07808 淮安分行风险部；07809 淮安分行零售部；07806 淮安分行公司部；07021 淮阴支行；07888 淮安分行清算中心；07999 淮安分行管理机构；D0601 涟水支行营业部大客户团队</v>
+        <v>07002 淮安分行财务部；06011 涟水支行；07013 淮安山阳分理处；07011 淮安区支行；07001 淮安分行营业部；07808 淮安分行风险部；07809 淮安分行零售部；07806 淮安分行公司部；07021 淮阴支行；07888 淮安分行清算中心；07999 淮安分行管理机构；A0701 淮安分行虚拟机构；A0702 淮安区支行 (空上级，逻辑上属 A0700)；A0703 涟水支行 (空上级，逻辑上属 A0700)；D0601 涟水支行营业部大客户团队</v>
       </c>
       <c r="K245" t="str">
         <v>A0000,A0700,A0800,A0900,A1000,A1100,A0400,A0500</v>
@@ -11909,7 +11909,7 @@
         <v>org_code='A0700'</v>
       </c>
       <c r="N245" t="str">
-        <v>org_code IN ('07002','06011','07013','07011','07001','07808','07809','07806','07021','07888','07999','D0601')</v>
+        <v>org_code IN ('07002','06011','07013','07011','07001','07808','07809','07806','07021','07888','07999','A0701','A0702','A0703','D0601')</v>
       </c>
       <c r="O245" t="str">
         <v/>
@@ -16359,10 +16359,10 @@
         <v/>
       </c>
       <c r="I340" t="str">
-        <v>02999,02011,02001,02031,02021,02041,02888,02111</v>
+        <v>B0001</v>
       </c>
       <c r="J340" t="str">
-        <v>02999 大丰村镇银行管理机构；02011 大丰港支行；02001 江苏大丰江南村镇银行股份有限公司；02031 裕华支行；02021 刘庄支行；02041 健康西路支行；02888 大丰村镇银行清算中心；02111 大丰小微贷款事业部</v>
+        <v>B0001 大丰村镇银行</v>
       </c>
       <c r="K340" t="str">
         <v>FR001,FR002,FR003</v>
@@ -16374,7 +16374,7 @@
         <v>org_code='FR002'</v>
       </c>
       <c r="N340" t="str">
-        <v>org_code IN ('02999','02011','02001','02031','02021','02041','02888','02111')</v>
+        <v>org_code IN ('B0001')</v>
       </c>
       <c r="O340" t="str">
         <v/>
@@ -16782,10 +16782,10 @@
         <v/>
       </c>
       <c r="I349" t="str">
-        <v/>
+        <v>02224,02225,02223,02222</v>
       </c>
       <c r="J349" t="str">
-        <v/>
+        <v>02224 大丰村行第三团队；02225 大丰村行第四团队；02223 大丰村行第二团队；02222 大丰村行第一团队</v>
       </c>
       <c r="K349" t="str">
         <v>02999,02011,02001,02031,02021,02041,02888,02111</v>
@@ -16797,7 +16797,7 @@
         <v>org_code='02111'</v>
       </c>
       <c r="N349" t="str">
-        <v/>
+        <v>org_code IN ('02224','02225','02223','02222')</v>
       </c>
       <c r="O349" t="str">
         <v/>
@@ -17017,10 +17017,10 @@
         <v/>
       </c>
       <c r="I354" t="str">
-        <v>03999,03011,03032,03021,03888,03001</v>
+        <v>C0001</v>
       </c>
       <c r="J354" t="str">
-        <v>03999 上海浦东江南村镇银行管理机构；03011 南汇支行；03032 普惠金融部团队；03021 三林支行；03888 上海浦东江南村镇银行清算中心；03001 上海浦东江南村镇银行营业部</v>
+        <v>C0001 上海浦东江南村镇银行</v>
       </c>
       <c r="K354" t="str">
         <v>FR001,FR002,FR003</v>
@@ -17032,7 +17032,7 @@
         <v>org_code='FR003'</v>
       </c>
       <c r="N354" t="str">
-        <v>org_code IN ('03999','03011','03032','03021','03888','03001')</v>
+        <v>org_code IN ('C0001')</v>
       </c>
       <c r="O354" t="str">
         <v/>
@@ -17393,10 +17393,10 @@
         <v/>
       </c>
       <c r="I362" t="str">
-        <v/>
+        <v>XN003</v>
       </c>
       <c r="J362" t="str">
-        <v/>
+        <v>XN003 丹阳农村商业银行不良资产经营部</v>
       </c>
       <c r="K362" t="str">
         <v>XN001,XN003</v>
@@ -17408,7 +17408,7 @@
         <v>org_code='XN001'</v>
       </c>
       <c r="N362" t="str">
-        <v/>
+        <v>org_code IN ('XN003')</v>
       </c>
       <c r="O362" t="str">
         <v/>
@@ -17440,10 +17440,10 @@
         <v/>
       </c>
       <c r="I363" t="str">
-        <v/>
+        <v>XN003</v>
       </c>
       <c r="J363" t="str">
-        <v/>
+        <v>XN003 丹阳农村商业银行不良资产经营部</v>
       </c>
       <c r="K363" t="str">
         <v>XN001,XN003</v>
@@ -17455,7 +17455,7 @@
         <v>org_code='XN001'</v>
       </c>
       <c r="N363" t="str">
-        <v/>
+        <v>org_code IN ('XN003')</v>
       </c>
       <c r="O363" t="str">
         <v/>
@@ -17487,10 +17487,10 @@
         <v/>
       </c>
       <c r="I364" t="str">
-        <v/>
+        <v>XN003</v>
       </c>
       <c r="J364" t="str">
-        <v/>
+        <v>XN003 丹阳农村商业银行不良资产经营部</v>
       </c>
       <c r="K364" t="str">
         <v>XN001,XN003</v>
@@ -17502,7 +17502,7 @@
         <v>org_code='XN001'</v>
       </c>
       <c r="N364" t="str">
-        <v/>
+        <v>org_code IN ('XN003')</v>
       </c>
       <c r="O364" t="str">
         <v/>
@@ -17694,7 +17694,7 @@
         <v>A0001-A0010 等</v>
       </c>
       <c r="D6" t="str">
-        <v>查本级: org_code='A0002'；下钻网点: 用 leaf_child_codes</v>
+        <v>查本级: org_code='A0002'；下钻下一级: 用 leaf_child_codes（仅直接子节点）</v>
       </c>
     </row>
     <row r="7">
@@ -17722,7 +17722,7 @@
         <v>D01xx</v>
       </c>
       <c r="D8" t="str">
-        <v>按 leaf_child_codes 或单码查询</v>
+        <v>按单码查询；父级 leaf_child_codes 含本团队</v>
       </c>
     </row>
     <row r="9">

</xml_diff>